<commit_message>
feat(tents): add optional contact_person field
Captures the contact person for exhibitors whose tent name is a company
or collective. Shown in the public SidePanel between the heading and
category badge when set; hidden when null. Surfaces in the admin
TentEditForm, Excel-Export column, and CSV/XLSX import wizard (incl. the
public import-template.xlsx). Migration adds a nullable text column on
tents - no data loss.

Import accepts the canonical 'contact_person' header plus the
'Ansprechperson' (DE) and 'Contact Person' aliases case-insensitively,
so admins don't have to rename their German spreadsheet columns.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/import-template.xlsx
+++ b/public/import-template.xlsx
@@ -397,46 +397,49 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:N2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
         <v>name</v>
       </c>
       <c r="B1" t="str">
+        <v>contact_person</v>
+      </c>
+      <c r="C1" t="str">
         <v>display_number</v>
       </c>
-      <c r="C1" t="str">
+      <c r="D1" t="str">
         <v>slug</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" t="str">
         <v>category_slugs</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>description_de</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>description_en</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>address</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>website_url</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>instagram_url</v>
       </c>
-      <c r="J1" t="str">
+      <c r="K1" t="str">
         <v>facebook_url</v>
       </c>
-      <c r="K1" t="str">
+      <c r="L1" t="str">
         <v>email_public</v>
       </c>
-      <c r="L1" t="str">
+      <c r="M1" t="str">
         <v>lat</v>
       </c>
-      <c r="M1" t="str">
+      <c r="N1" t="str">
         <v>lng</v>
       </c>
     </row>
@@ -444,29 +447,29 @@
       <c r="A2" t="str">
         <v>Galerie Müller</v>
       </c>
-      <c r="B2">
+      <c r="B2" t="str">
+        <v>Anna Müller</v>
+      </c>
+      <c r="C2">
         <v>42</v>
       </c>
-      <c r="C2" t="str">
+      <c r="D2" t="str">
         <v/>
       </c>
-      <c r="D2" t="str">
+      <c r="E2" t="str">
         <v>painting</v>
       </c>
-      <c r="E2" t="str">
+      <c r="F2" t="str">
         <v>Zeitgenössische Malerei</v>
       </c>
-      <c r="F2" t="str">
+      <c r="G2" t="str">
         <v>Contemporary painting</v>
       </c>
-      <c r="G2" t="str">
+      <c r="H2" t="str">
         <v>Hauptstraße 1</v>
       </c>
-      <c r="H2" t="str">
+      <c r="I2" t="str">
         <v>https://example.com</v>
-      </c>
-      <c r="I2" t="str">
-        <v/>
       </c>
       <c r="J2" t="str">
         <v/>
@@ -474,16 +477,19 @@
       <c r="K2" t="str">
         <v/>
       </c>
-      <c r="L2">
+      <c r="L2" t="str">
+        <v/>
+      </c>
+      <c r="M2">
         <v>49</v>
       </c>
-      <c r="M2">
+      <c r="N2">
         <v>8.4</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(tents): add optional contact_person field (#32)
Captures the contact person for exhibitors whose tent name is a company
or collective. Shown in the public SidePanel between the heading and
category badge when set; hidden when null. Surfaces in the admin
TentEditForm, Excel-Export column, and CSV/XLSX import wizard (incl. the
public import-template.xlsx). Migration adds a nullable text column on
tents - no data loss.

Import accepts the canonical 'contact_person' header plus the
'Ansprechperson' (DE) and 'Contact Person' aliases case-insensitively,
so admins don't have to rename their German spreadsheet columns.

Co-authored-by: Jan Poepke <jpoepke@gmail.com>
Co-authored-by: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/import-template.xlsx
+++ b/public/import-template.xlsx
@@ -397,46 +397,49 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:N2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
         <v>name</v>
       </c>
       <c r="B1" t="str">
+        <v>contact_person</v>
+      </c>
+      <c r="C1" t="str">
         <v>display_number</v>
       </c>
-      <c r="C1" t="str">
+      <c r="D1" t="str">
         <v>slug</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" t="str">
         <v>category_slugs</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>description_de</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>description_en</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>address</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>website_url</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>instagram_url</v>
       </c>
-      <c r="J1" t="str">
+      <c r="K1" t="str">
         <v>facebook_url</v>
       </c>
-      <c r="K1" t="str">
+      <c r="L1" t="str">
         <v>email_public</v>
       </c>
-      <c r="L1" t="str">
+      <c r="M1" t="str">
         <v>lat</v>
       </c>
-      <c r="M1" t="str">
+      <c r="N1" t="str">
         <v>lng</v>
       </c>
     </row>
@@ -444,29 +447,29 @@
       <c r="A2" t="str">
         <v>Galerie Müller</v>
       </c>
-      <c r="B2">
+      <c r="B2" t="str">
+        <v>Anna Müller</v>
+      </c>
+      <c r="C2">
         <v>42</v>
       </c>
-      <c r="C2" t="str">
+      <c r="D2" t="str">
         <v/>
       </c>
-      <c r="D2" t="str">
+      <c r="E2" t="str">
         <v>painting</v>
       </c>
-      <c r="E2" t="str">
+      <c r="F2" t="str">
         <v>Zeitgenössische Malerei</v>
       </c>
-      <c r="F2" t="str">
+      <c r="G2" t="str">
         <v>Contemporary painting</v>
       </c>
-      <c r="G2" t="str">
+      <c r="H2" t="str">
         <v>Hauptstraße 1</v>
       </c>
-      <c r="H2" t="str">
+      <c r="I2" t="str">
         <v>https://example.com</v>
-      </c>
-      <c r="I2" t="str">
-        <v/>
       </c>
       <c r="J2" t="str">
         <v/>
@@ -474,16 +477,19 @@
       <c r="K2" t="str">
         <v/>
       </c>
-      <c r="L2">
+      <c r="L2" t="str">
+        <v/>
+      </c>
+      <c r="M2">
         <v>49</v>
       </c>
-      <c r="M2">
+      <c r="N2">
         <v>8.4</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add internal phone number to tents
Admins can record an internal contact phone per tent. It mirrors the email_public pattern: editable in the admin form, round-trips through CSV/XLSX import, and is written into the static HTML export, but is deliberately NOT rendered in the public SidePanel (a guard test locks this in).

Adds: migration (tents.phone text), supabase types, RHF field + DE/EN i18n labels, persist in TentEditPage, import mapping + Telefon/Phone header aliases, export column (last) + regenerated import-template.xlsx, and the HTML export field.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/import-template.xlsx
+++ b/public/import-template.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:O2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -442,6 +442,9 @@
       <c r="N1" t="str">
         <v>lng</v>
       </c>
+      <c r="O1" t="str">
+        <v>phone</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -486,10 +489,13 @@
       <c r="N2">
         <v>8.4</v>
       </c>
+      <c r="O2" t="str">
+        <v>+49 4141 123456</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>